<commit_message>
Lead QA demos with three longer manual advisor journeys
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qa/Wealth-Platform-Manual-QA.xlsx
+++ b/qa/Wealth-Platform-Manual-QA.xlsx
@@ -13,13 +13,13 @@
     <sheet name="Execution Guide" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$K$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$K$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Test Cases'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Steps'!$A$1:$F$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Steps'!$A$1:$F$257</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Steps'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements Traceability'!$A$1:$F$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Requirements Traceability'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Execution Guide'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Execution Guide'!$A$1:$B$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Execution Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3289,8 +3289,173 @@
         <v>6</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>https://cognition-team-x9dqnayp.atlassian.net/browse/KAN-12</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Restore the deterministic synthetic seed with the controlled harness before this case. Start at /?screen=workspace&amp;area=clients. Perform this as one uninterrupted advisor journey; assert every expected result and use journeyStep for a 1.5-second reading hold after each meaningful step.</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>C1002 James Chen; A1003 Chen USD Investment; MSFT 40 shares; risk Conservative to Moderate; KYC Review due to Current.</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>https://cognition-team-x9dqnayp.atlassian.net/browse/KAN-14</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Restore the deterministic synthetic seed with the controlled harness before this case. Start at /?screen=workspace&amp;area=clients. Perform this as one uninterrupted advisor journey; assert every expected result and use journeyStep for a 1.5-second reading hold after each meaningful step.</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>C1001 Eleanor Whitfield; A1001 Whitfield Investment; RY 100 shares at CAD 140.00; buy 10 shares for CAD 1,400.00; cash CAD 25,000.00.</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Move Money</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>https://cognition-team-x9dqnayp.atlassian.net/browse/KAN-15</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Restore the deterministic synthetic seed with the controlled harness before this case. Start at /?screen=workspace&amp;area=clients. Perform this as one uninterrupted advisor journey; assert every expected result and use journeyStep for a 1.5-second reading hold after each meaningful step.</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>C1001 Eleanor Whitfield; from A1001 CAD 25,000.00 to A1002 CAD 10,000.00; initial amount 1,000.00 amended to 1,250.00; reference Quarterly cash allocation.</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K51"/>
+  <autoFilter ref="A1:K54"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
@@ -3392,6 +3557,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId106"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
@@ -3404,7 +3575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F212"/>
+  <dimension ref="A1:F257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9777,8 +9948,1358 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Click Search clients and enter C1002.</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>Only James Chen (C1002) remains in the client book.</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Click Filter by KYC status and choose Review due.</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>James Chen remains visible with Conservative risk and Review due KYC.</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Click James Chen in the client book.</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>The detail panel identifies C1002 and shows only A1003, USD 15,000.00 cash.</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Click Edit profile.</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>The editable profile form shows Conservative risk and Review due KYC.</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Click the Risk profile field and choose Moderate.</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>The draft risk is Moderate; the saved profile still shows Conservative.</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Click the KYC status field and choose Current.</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>The draft KYC is Current; the saved profile still shows Review due.</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Click Save profile.</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>A success notice confirms James Chen, Moderate risk and Current KYC. The detail panel shows the saved values, even if the Review due filter now hides the client row.</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Click View portfolio.</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio opens scoped to James Chen, not another client.</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Click Account and choose A1003 Chen USD Investment.</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>Only A1003 holdings are shown; MSFT quantity is 40 and market value is USD 16,800.00.</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Click Instrument and choose MSFT.</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>Only the MSFT holding in A1003 is shown, with quantity 40 and USD currency.</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Click the Clients workspace tab.</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>The client book reopens.</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Click James Chen in the client book.</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>The detail panel shows Moderate risk, Current KYC and the same A1003 account.</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Click Refresh data.</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>Moderate risk and Current KYC remain saved; Eleanor Whitfield remains Moderate and Current.</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-051</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Complete a client review from KYC search to saved profile and portfolio</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Click Edit profile to inspect the saved fields, then click Cancel.</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>The form defaults to Moderate and Current; cancelling makes no additional change. The client detail and USD 15,000.00 cash remain unchanged.</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>KAN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Click Search clients and enter C1001.</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>Only Eleanor Whitfield appears.</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Click Eleanor Whitfield, then click View portfolio.</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio is scoped to C1001 and shows only her CAD accounts.</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Click Account and choose A1001.</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>RY quantity is 100; cash is CAD 25,000.00 and no cash is reserved.</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Click the Orders workspace tab.</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>The new-order ticket and empty order blotter appear.</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Click Account and choose A1001 Whitfield Investment.</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>The ticket is scoped to the CAD account and available cash is CAD 25,000.00.</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Click Instrument and choose RY.</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>The indicative price is CAD 140.00 and held quantity is 100 RY.</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Click Buy, then click Quantity and enter 10.</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>Buy is selected and estimated value is CAD 1,400.00; no order exists yet.</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Click Place order.</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one Open buy for 10 RY appears. Available cash becomes CAD 23,600.00; held quantity remains 100.</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>Click Order status and choose Open.</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>The new Open order remains visible.</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Click Search orders and enter RY.</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>The same order is visible with account A1001, quantity 10 and value CAD 1,400.00.</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Click Cancel order on that row.</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>The order becomes Cancelled and disappears from the Open filter.</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Click Order status and choose Cancelled.</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>The cancelled order is visible with the same ID and quantity. No second order was created.</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>Click the Portfolio workspace tab.</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio opens for a fresh account review.</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Click Client and choose C1001; click Account and choose A1001.</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>RY quantity remains 100; cash and available cash are CAD 25,000.00 and reserved cash is zero.</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-052</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Review a holding, place a buy order and verify cancellation releases cash</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Click Refresh data.</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>The released cash and unchanged 100-share holding persist after a server refresh.</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>KAN-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Click Search clients and enter C1001, then click Eleanor Whitfield.</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>The detail panel shows A1001 cash CAD 25,000.00 and A1002 cash CAD 10,000.00.</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>Click View portfolio.</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio opens scoped to Eleanor Whitfield.</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Click Account and choose A1001.</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>The investment account shows CAD 25,000.00 cash and 100 RY shares.</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Click the Move Money workspace tab.</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>An empty new-transfer form and empty transfer history appear.</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Click From account and choose A1001.</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>Only eligible same-client CAD destination accounts can be selected.</t>
+        </is>
+      </c>
+      <c r="F246" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>Click To account and choose A1002.</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>Whitfield Savings is selected; A1001 and Chen's USD account are not eligible destinations.</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Click Amount (CAD) and enter 1000.00.</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>The draft amount is 1000.00; no transfer exists and no money has moved.</t>
+        </is>
+      </c>
+      <c r="F248" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Click Reference and enter Quarterly cash allocation.</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>The reference is visible in the draft.</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Click Review transfer.</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>The review identifies Eleanor, A1001 to A1002, CAD 1,000.00 and the reference; no transfer is committed.</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>Click Edit transfer.</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>The original account, amount and reference values remain available for editing.</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>Click Amount (CAD) and replace it with 1250.00.</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>The revised draft is CAD 1,250.00 and no transfer exists.</t>
+        </is>
+      </c>
+      <c r="F252" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>Click Review transfer again.</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>The review shows CAD 1,250.00 with the same source, destination and reference.</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Click Confirm transfer.</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one Completed transfer for CAD 1,250.00 appears, not a separate CAD 1,000.00 transfer.</t>
+        </is>
+      </c>
+      <c r="F254" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>Click Search transfers and enter Quarterly cash allocation.</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>Exactly that completed transfer is shown with A1001 as source and A1002 as destination.</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>Click the Clients workspace tab, then click Eleanor Whitfield.</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>A1001 cash is CAD 23,750.00 and A1002 cash is CAD 11,250.00; combined cash remains CAD 35,000.00.</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>WM-TC-053</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Review, amend and confirm a cash transfer then reconcile client balances</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>Click Refresh data.</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>Both balances persist and combined cash is conserved; no duplicate transfer is created.</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr">
+        <is>
+          <t>KAN-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F212"/>
+  <autoFilter ref="A1:F257"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -9991,6 +11512,51 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId209"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId256"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
@@ -10063,11 +11629,11 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>WM-TC-001, WM-TC-002, WM-TC-003, WM-TC-004, WM-TC-005, WM-TC-006, WM-TC-007, WM-TC-008</t>
+          <t>WM-TC-001, WM-TC-002, WM-TC-003, WM-TC-004, WM-TC-005, WM-TC-006, WM-TC-007, WM-TC-008, WM-TC-051</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -10123,11 +11689,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>WM-TC-019, WM-TC-020, WM-TC-021, WM-TC-022, WM-TC-023, WM-TC-024, WM-TC-025, WM-TC-026, WM-TC-027, WM-TC-028, WM-TC-029, WM-TC-030</t>
+          <t>WM-TC-019, WM-TC-020, WM-TC-021, WM-TC-022, WM-TC-023, WM-TC-024, WM-TC-025, WM-TC-026, WM-TC-027, WM-TC-028, WM-TC-029, WM-TC-030, WM-TC-052</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -10153,11 +11719,11 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>WM-TC-031, WM-TC-032, WM-TC-033, WM-TC-034, WM-TC-035, WM-TC-036, WM-TC-037, WM-TC-038</t>
+          <t>WM-TC-031, WM-TC-032, WM-TC-033, WM-TC-034, WM-TC-035, WM-TC-036, WM-TC-037, WM-TC-038, WM-TC-053</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -10253,7 +11819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10275,161 +11841,173 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>Opening advisor journeys</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Manual UAT cases for the synthetic Wealth Platform connected workspace demo. All clients, accounts, balances and exceptions are fictional sandbox data; no real RBC customer data is used.</t>
+          <t>53 manual cases: the original WM-TC-001..050 are unchanged, plus WM-TC-051 client review (Clients), WM-TC-052 buy/cancel (Orders), WM-TC-053 amend/confirm transfer (Move Money). Author these from the spreadsheet like every other case. Their baseline recordings lead the composite video in that order. Each starts in Clients and follows 10+ meaningful clicks across screens. Use journeyStep with assertions and 1.5-second reading holds; visibly click fields before typing/selecting. Preserve one uninterrupted recording per journey. Wiki-derived gaps remain separate.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Application URL</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Open &lt;base URL&gt;/?screen=workspace&amp;area=&lt;area&gt;, where area is clients, portfolio, orders, money, rebalance or settlements. Each case names the area to start from.</t>
+          <t>Manual UAT cases for the synthetic Wealth Platform connected workspace demo. All clients, accounts, balances and exceptions are fictional sandbox data; no real RBC customer data is used.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Reset before every case</t>
+          <t>Application URL</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Before starting each case, restore the deterministic seed using the controlled test harness reset supplied by the test lead. Do not use any in-app reset control. Then reload the browser so it shows the seeded state.</t>
+          <t>Open &lt;base URL&gt;/?screen=workspace&amp;area=&lt;area&gt;, where area is clients, portfolio, orders, money, rebalance or settlements. Each case names the area to start from.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Seed: clients</t>
+          <t>Reset before every case</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>C1001 Eleanor Whitfield, risk Moderate, KYC Current. C1002 James Chen, risk Conservative, KYC Review due.</t>
+          <t>Before starting each case, restore the deterministic seed using the controlled test harness reset supplied by the test lead. Do not use any in-app reset control. Then reload the browser so it shows the seeded state.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Seed: accounts</t>
+          <t>Seed: clients</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A1001 Whitfield Investment (C1001), CAD 25,000.00 cash. A1002 Whitfield Savings (C1001), CAD 10,000.00 cash. A1003 Chen USD Investment (C1002), USD 15,000.00 cash.</t>
+          <t>C1001 Eleanor Whitfield, risk Moderate, KYC Current. C1002 James Chen, risk Conservative, KYC Review due.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Seed: positions</t>
+          <t>Seed: accounts</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>P1001 A1001 RY Royal Bank of Canada 100 @ 140.00 CAD (14,000.00). P1002 A1002 BMO 80 @ 125.00 CAD (10,000.00). P1003 A1003 MSFT 40 @ 420.00 USD (16,800.00).</t>
+          <t>A1001 Whitfield Investment (C1001), CAD 25,000.00 cash. A1002 Whitfield Savings (C1001), CAD 10,000.00 cash. A1003 Chen USD Investment (C1002), USD 15,000.00 cash.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Seed: orders and transfers</t>
+          <t>Seed: positions</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>No orders and no transfers exist at seed. Any order or transfer a case needs is created through the UI inside that case.</t>
+          <t>P1001 A1001 RY Royal Bank of Canada 100 @ 140.00 CAD (14,000.00). P1002 A1002 BMO 80 @ 125.00 CAD (10,000.00). P1003 A1003 MSFT 40 @ 420.00 USD (16,800.00).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Seed: model targets</t>
+          <t>Seed: orders and transfers</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Equity 60%, Fixed income 30%, Cash 10%; current allocation equals targets at seed.</t>
+          <t>No orders and no transfers exist at seed. Any order or transfer a case needs is created through the UI inside that case.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Seed: settlement exceptions</t>
+          <t>Seed: model targets</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>EX1001 A1001 Missing settlement instructions, Open, unassigned. EX1002 A1003 Cash reconciliation, Open, unassigned. Assignable owners: A. Nguyen, S. Patel.</t>
+          <t>Equity 60%, Fixed income 30%, Cash 10%; current allocation equals targets at seed.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Executing steps</t>
+          <t>Seed: settlement exceptions</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perform every step in the browser exactly as written and compare the screen against the expected result for that step. Record Pass or Fail per step; a case passes only if every step passes.</t>
+          <t>EX1001 A1001 Missing settlement instructions, Open, unassigned. EX1002 A1003 Cash reconciliation, Open, unassigned. Assignable owners: A. Nguyen, S. Patel.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Invalid input checks</t>
+          <t>Executing steps</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Where a step expects a rejection, confirm that a clear error is shown AND that no record, balance, holding, status or audit entry changed, including after a browser reload.</t>
+          <t>Perform every step in the browser exactly as written and compare the screen against the expected result for that step. Record Pass or Fail per step; a case passes only if every step passes.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>Invalid input checks</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Capture a screenshot of the final expected state and of any failure. Note the case Id, step number, observed result and timestamp in the defect or run record.</t>
+          <t>Where a step expects a rejection, confirm that a clear error is shown AND that no record, balance, holding, status or audit entry changed, including after a browser reload.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Capture a screenshot of the final expected state and of any failure. Note the case Id, step number, observed result and timestamp in the defect or run record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Traceability</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Each case links to its Jira story in the Requirements Traceability sheet and the Requirement column. This workbook follows a qTest-style export layout for review; it is not a certified qTest import file.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>